<commit_message>
Faz 6 / 6h: grafik ve resim .xlsx okuma/yazma, Tabcel imi, Excel doğrulama aracı
- io/xlsx_grafik.py: 7 tür x alt tür yazma/okuma, resim kayıpsız, TabcelSurum imi, autoTitleDeleted
- uyarı mantığı: im yoksa "uyarlandı", desteklenmeyen tür/seri atlanır ve bildirilir
- openpyxl AreaChart axId hatası giderildi
- gerçek Excel (COM) ile doğrulandı: araclar/excel_dogrula.ps1; başlık/gösterge binmesi ve siyah ızgara düzeltildi
- test_xlsx_grafik.py (33), grafikli.xlsx örneği gerçek resimle yeniden üretildi, grafikli test güncellendi
- yardım, CLAUDE.md (Excel kurulu), surec.md güncellendi

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testler/ornekler/grafikli.xlsx
+++ b/testler/ornekler/grafikli.xlsx
@@ -257,6 +257,31 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 

</xml_diff>